<commit_message>
Better detection of overlaps
</commit_message>
<xml_diff>
--- a/activityAnalysis/Appointments_to_database.xlsx
+++ b/activityAnalysis/Appointments_to_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rachaelnaphtal/Documents/JudgingAnalysis/activityAnalysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C561D6CC-A56E-A84F-8181-49CDFCBA9E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDC8553-8194-9C46-87DA-0EE56371CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14180" yWindow="760" windowWidth="14420" windowHeight="17020" xr2:uid="{3DC34758-EE40-AE44-9218-4BCDC75CCCC4}"/>
+    <workbookView xWindow="3040" yWindow="760" windowWidth="14420" windowHeight="17020" xr2:uid="{3DC34758-EE40-AE44-9218-4BCDC75CCCC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="260">
   <si>
     <t>Position</t>
   </si>
@@ -836,6 +836,12 @@
   </si>
   <si>
     <t>Chief TA</t>
+  </si>
+  <si>
+    <t>J-SYS</t>
+  </si>
+  <si>
+    <t>R-SYS</t>
   </si>
 </sst>
 </file>
@@ -1247,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02FBD72-4F6F-8A41-B8B8-FF6C38999B4C}">
-  <dimension ref="A1:F324"/>
+  <dimension ref="A1:F326"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -5505,6 +5511,28 @@
       </c>
       <c r="E324">
         <v>7</v>
+      </c>
+    </row>
+    <row r="325" spans="1:6">
+      <c r="A325" t="s">
+        <v>258</v>
+      </c>
+      <c r="C325">
+        <v>1</v>
+      </c>
+      <c r="E325">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="326" spans="1:6">
+      <c r="A326" t="s">
+        <v>259</v>
+      </c>
+      <c r="C326">
+        <v>4</v>
+      </c>
+      <c r="E326">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>